<commit_message>
Improve data uploading with processing details and progress tracking
Refactors test upload script to ES modules, adjusts port configurations and file paths.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 0742d766-0a68-4246-b1c6-4bcdb589d357
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/e20af904-8583-409a-8a9e-51ad07e0801f/56fef072-77c7-4856-b3e1-96fcdac5842b.jpg
</commit_message>
<xml_diff>
--- a/test_observations.xlsx
+++ b/test_observations.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Validated Observations" sheetId="1" r:id="rId1"/>
+    <sheet name="Test Observations" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,161 +397,151 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:K4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Observation ID</v>
+        <v>Reference Number</v>
       </c>
       <c r="B1" t="str">
-        <v>Scientific Name</v>
+        <v>Source Database</v>
       </c>
       <c r="C1" t="str">
-        <v>Common Name</v>
+        <v>Genus</v>
       </c>
       <c r="D1" t="str">
-        <v>Phylum</v>
+        <v>Species</v>
       </c>
       <c r="E1" t="str">
-        <v>Class</v>
+        <v>Collector</v>
       </c>
       <c r="F1" t="str">
-        <v>Order</v>
+        <v>Report Date</v>
       </c>
       <c r="G1" t="str">
-        <v>Family</v>
+        <v>Country</v>
       </c>
       <c r="H1" t="str">
-        <v>Genus</v>
+        <v>State</v>
       </c>
       <c r="I1" t="str">
-        <v>Species</v>
+        <v>City</v>
       </c>
       <c r="J1" t="str">
         <v>Latitude</v>
       </c>
       <c r="K1" t="str">
         <v>Longitude</v>
-      </c>
-      <c r="L1" t="str">
-        <v>State</v>
-      </c>
-      <c r="M1" t="str">
-        <v>Observed On</v>
-      </c>
-      <c r="N1" t="str">
-        <v>Observer</v>
-      </c>
-      <c r="O1" t="str">
-        <v>Collector</v>
-      </c>
-      <c r="P1" t="str">
-        <v>Institution</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>TEST001</v>
+        <v>265571056</v>
       </c>
       <c r="B2" t="str">
-        <v>Agaricus bisporus</v>
+        <v>iNaturalist</v>
       </c>
       <c r="C2" t="str">
-        <v>Button Mushroom</v>
+        <v>Amanita</v>
       </c>
       <c r="D2" t="str">
-        <v>Basidiomycota</v>
+        <v>Amanita muscaria</v>
       </c>
       <c r="E2" t="str">
-        <v>Agaricomycetes</v>
+        <v>Test Collector</v>
       </c>
       <c r="F2" t="str">
-        <v>Agaricales</v>
+        <v>2024-01-15</v>
       </c>
       <c r="G2" t="str">
-        <v>Agaricaceae</v>
+        <v>United States</v>
       </c>
       <c r="H2" t="str">
-        <v>Agaricus</v>
+        <v>California</v>
       </c>
       <c r="I2" t="str">
-        <v>bisporus</v>
+        <v>San Francisco</v>
       </c>
       <c r="J2" t="str">
-        <v>40.7128</v>
+        <v>37.7749</v>
       </c>
       <c r="K2" t="str">
-        <v>-74.0060</v>
-      </c>
-      <c r="L2" t="str">
-        <v>New York</v>
-      </c>
-      <c r="M2" t="str">
-        <v>2024-05-15</v>
-      </c>
-      <c r="N2" t="str">
-        <v>Test Observer</v>
-      </c>
-      <c r="O2" t="str">
-        <v>Test Collector</v>
-      </c>
-      <c r="P2" t="str">
-        <v>Test University</v>
+        <v>-122.4194</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>TEST002</v>
+        <v>123456789</v>
       </c>
       <c r="B3" t="str">
-        <v>Pleurotus ostreatus</v>
+        <v>iNaturalist</v>
       </c>
       <c r="C3" t="str">
-        <v>Oyster Mushroom</v>
+        <v>Boletus</v>
       </c>
       <c r="D3" t="str">
-        <v>Basidiomycota</v>
+        <v>Boletus edulis</v>
       </c>
       <c r="E3" t="str">
-        <v>Agaricomycetes</v>
+        <v>Another Collector</v>
       </c>
       <c r="F3" t="str">
-        <v>Agaricales</v>
+        <v>2024-02-10</v>
       </c>
       <c r="G3" t="str">
-        <v>Pleurotaceae</v>
+        <v>United States</v>
       </c>
       <c r="H3" t="str">
-        <v>Pleurotus</v>
+        <v>Oregon</v>
       </c>
       <c r="I3" t="str">
-        <v>ostreatus</v>
+        <v>Portland</v>
       </c>
       <c r="J3" t="str">
-        <v>34.0522</v>
+        <v>45.5152</v>
       </c>
       <c r="K3" t="str">
-        <v>-118.2437</v>
-      </c>
-      <c r="L3" t="str">
-        <v>California</v>
-      </c>
-      <c r="M3" t="str">
-        <v>2024-05-20</v>
-      </c>
-      <c r="N3" t="str">
-        <v>Test Observer 2</v>
-      </c>
-      <c r="O3" t="str">
-        <v>Test Collector 2</v>
-      </c>
-      <c r="P3" t="str">
-        <v>Test Institute</v>
+        <v>-122.6784</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>987654321</v>
+      </c>
+      <c r="B4" t="str">
+        <v>iNaturalist</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Cantharellus</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Cantharellus cibarius</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Test User</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2024-03-05</v>
+      </c>
+      <c r="G4" t="str">
+        <v>United States</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Washington</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Seattle</v>
+      </c>
+      <c r="J4" t="str">
+        <v>47.6062</v>
+      </c>
+      <c r="K4" t="str">
+        <v>-122.3321</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>